<commit_message>
[02/10/2026] Updates financial data research
</commit_message>
<xml_diff>
--- a/data/data-source-checklist.xlsx
+++ b/data/data-source-checklist.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="45">
   <si>
     <t>Year</t>
   </si>
@@ -48,18 +48,30 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Idioma</t>
+  </si>
+  <si>
     <t>2020_Financialdocuments-December31,2020</t>
   </si>
   <si>
     <t>31/12/2020</t>
   </si>
   <si>
+    <t>EN</t>
+  </si>
+  <si>
     <t>2021_Financialdocuments-December31,2021</t>
   </si>
   <si>
     <t>31/12/2021</t>
   </si>
   <si>
+    <t>2022_Financialdocuments-December31,2022</t>
+  </si>
+  <si>
+    <t>31/12/2022</t>
+  </si>
+  <si>
     <t>2023_Financialdocuments-December31,2023</t>
   </si>
   <si>
@@ -106,13 +118,43 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>2020_Results_Financial_Document</t>
+  </si>
+  <si>
+    <t>31/12/2026</t>
+  </si>
+  <si>
+    <t>2021_Results_Financial_Document</t>
+  </si>
+  <si>
+    <t>2022_Results_Financial_Document</t>
+  </si>
+  <si>
+    <t>2024_Kering_Document_financier</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>p. 40</t>
+  </si>
+  <si>
+    <t>p. 42</t>
+  </si>
+  <si>
+    <t>p. 43</t>
+  </si>
+  <si>
+    <t>2025_Results_Financial_Document</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -136,8 +178,18 @@
       <color rgb="FF000100"/>
       <sz val="10"/>
     </font>
+    <font>
+      <color rgb="FF2C3E50"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <color rgb="FF2C3E50"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -164,31 +216,6 @@
         <fgColor rgb="FFFE0000"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4BFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF7FF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0007FF"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -202,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom"/>
@@ -220,12 +247,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -249,16 +270,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -651,7 +681,9 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2"/>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
@@ -678,12 +710,14 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L2" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
@@ -710,12 +744,14 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -733,17 +769,23 @@
       <c r="A4" s="3">
         <v>2022</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -770,12 +812,14 @@
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="L5" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -794,7 +838,7 @@
         <v>2024</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -804,12 +848,14 @@
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L6" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -828,28 +874,30 @@
         <v>2025</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="9"/>
+      <c r="I7" s="7"/>
       <c r="J7" s="6" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L7" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -870,7 +918,7 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -894,8 +942,8 @@
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
-      <c r="C9" s="10" t="s">
-        <v>26</v>
+      <c r="C9" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -922,8 +970,8 @@
     <row r="10" ht="12.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
-      <c r="C10" s="11" t="s">
-        <v>27</v>
+      <c r="C10" s="9" t="s">
+        <v>31</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -950,8 +998,8 @@
     <row r="11" ht="12.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
-      <c r="C11" s="12" t="s">
-        <v>28</v>
+      <c r="C11" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -978,8 +1026,8 @@
     <row r="12" ht="12.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
-      <c r="C12" s="13" t="s">
-        <v>29</v>
+      <c r="C12" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1007,7 +1055,7 @@
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -1065,9 +1113,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
@@ -1743,7 +1789,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="9.285714285714286" customWidth="1"/>
@@ -1758,104 +1804,209 @@
     <col min="12" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="12.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" ht="12.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
+      <c r="L1" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" ht="12.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="13">
         <v>2020</v>
       </c>
-    </row>
-    <row r="3" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" ht="12.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="13">
         <v>2021</v>
       </c>
-    </row>
-    <row r="4" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" ht="12.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="13">
         <v>2022</v>
       </c>
-    </row>
-    <row r="5" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15">
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" ht="12.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="13">
         <v>2023</v>
       </c>
-    </row>
-    <row r="6" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+    </row>
+    <row r="6" ht="12.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="13">
         <v>2024</v>
       </c>
-    </row>
-    <row r="7" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" ht="12.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="13">
         <v>2025</v>
       </c>
+      <c r="B7" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="K7" t="s">
+        <v>28</v>
+      </c>
+      <c r="L7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="9" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="16" t="s">
-        <v>26</v>
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="18" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="17" t="s">
-        <v>27</v>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="19" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="18" t="s">
-        <v>28</v>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="20" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="19" t="s">
-        <v>29</v>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="21" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15" t="s">
-        <v>30</v>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="22" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1882,103 +2033,103 @@
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="12" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
+      <c r="A2" s="13">
         <v>2020</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15">
+      <c r="A3" s="13">
         <v>2021</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="A4" s="13">
         <v>2022</v>
       </c>
     </row>
     <row r="5" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15">
+      <c r="A5" s="13">
         <v>2023</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
+      <c r="A6" s="13">
         <v>2024</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+      <c r="A7" s="13">
         <v>2025</v>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="16" t="s">
-        <v>26</v>
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="18" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="17" t="s">
-        <v>27</v>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="19" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="18" t="s">
-        <v>28</v>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="20" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="19" t="s">
-        <v>29</v>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="21" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15" t="s">
-        <v>30</v>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="22" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>